<commit_message>
move and add files
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/SecondaryCareAnalysis/OP/Overall/Output_Costs_Raw.xlsx
+++ b/CPRD Raw Analysis/Results/SecondaryCareAnalysis/OP/Overall/Output_Costs_Raw.xlsx
@@ -417,34 +417,34 @@
         <v>20691</v>
       </c>
       <c r="B2">
-        <v>1339.19</v>
+        <v>1372.39</v>
       </c>
       <c r="C2">
-        <v>31.46</v>
+        <v>12.88</v>
       </c>
       <c r="D2">
-        <v>77425.78</v>
+        <v>39989.81</v>
       </c>
       <c r="E2">
-        <v>1750.14</v>
+        <v>1700.11</v>
       </c>
       <c r="F2">
-        <v>874.6799999999999</v>
+        <v>874.33</v>
       </c>
       <c r="G2">
-        <v>490.13</v>
+        <v>435.68</v>
       </c>
       <c r="H2">
-        <v>1638.42</v>
+        <v>1703.14</v>
       </c>
       <c r="I2">
-        <v>12.17</v>
+        <v>11.82</v>
       </c>
       <c r="J2">
-        <v>1315.34</v>
+        <v>1349.22</v>
       </c>
       <c r="K2">
-        <v>1363.04</v>
+        <v>1395.55</v>
       </c>
     </row>
   </sheetData>
@@ -519,34 +519,34 @@
         <v>23106</v>
       </c>
       <c r="B2">
-        <v>1199.1</v>
+        <v>1228.75</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>77425.78</v>
+        <v>39989.81</v>
       </c>
       <c r="E2">
-        <v>1706.04</v>
+        <v>1662.63</v>
       </c>
       <c r="F2">
-        <v>766.33</v>
+        <v>748.47</v>
       </c>
       <c r="G2">
-        <v>354.3</v>
+        <v>323.24</v>
       </c>
       <c r="H2">
-        <v>1506.82</v>
+        <v>1562.39</v>
       </c>
       <c r="I2">
-        <v>11.22</v>
+        <v>10.94</v>
       </c>
       <c r="J2">
-        <v>1177.1</v>
+        <v>1207.31</v>
       </c>
       <c r="K2">
-        <v>1221.1</v>
+        <v>1250.19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>